<commit_message>
Prove grouped all-error pivot rankings and lookups
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/ExcelPivotCorpus/AllErrorRanking/bottom-average.xlsx
+++ b/OfficeIMO.TestAssets/Documents/ExcelPivotCorpus/AllErrorRanking/bottom-average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\przemyslaw.klys.EVOTEC\.codex\worktrees\excel-csv-quality\OfficeIMO\OfficeIMO.TestAssets\Documents\ExcelPivotCorpus\AllErrorRanking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{595724E1-1CD9-40D5-9B03-5B9CD7E2237F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{949B1E22-1AEB-4072-B8E1-3E4FD0010377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="16170" windowWidth="28996" windowHeight="15675" xr2:uid="{892B5326-F570-460C-9E04-F0AA908A72EC}"/>
+    <workbookView xWindow="-98" yWindow="16170" windowWidth="28996" windowHeight="15675" xr2:uid="{8573BB1B-A9DC-4ED2-AA9A-B8284ADFB2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Grouped" sheetId="2" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="OfficeIMO Word COM Fixture" refreshedDate="46293.576872106481" createdVersion="6" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{161DF8F7-4A89-4FC4-970D-99E09321C4CA}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="OfficeIMO Word COM Fixture" refreshedDate="46293.579433796294" createdVersion="6" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{97AFF336-2A8A-4519-A6C0-E6316255AE2A}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:B4" sheet="Source"/>
   </cacheSource>
@@ -164,7 +164,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9E06337F-EA94-4F10-BDBC-EFB34CD4C211}" name="AllErrorPivot" cacheId="79" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{67C70C15-C44E-4D45-BCA5-8B6354840DA8}" name="AllErrorPivot" cacheId="79" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A4:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" measureFilter="1">
@@ -531,7 +531,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BC513D3-9163-4475-A5DE-572C2180A97E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1F2708D-F3F1-40F5-821E-F7A49CDA7665}">
   <dimension ref="A4:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -569,7 +569,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE1A4BE0-E83C-41F6-9CFD-E9A0A1A629ED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E6E2C01-FBC7-4661-BDA1-E1D5D5A65606}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>

</xml_diff>